<commit_message>
Add submodule dataprocessor table description
</commit_message>
<xml_diff>
--- a/R-dataprocessor/submodules/Dataprocessor_Submodules_Table_Description.xlsx
+++ b/R-dataprocessor/submodules/Dataprocessor_Submodules_Table_Description.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="44">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -124,6 +124,12 @@
     <t xml:space="preserve">optional – Redcap repeat instance id</t>
   </si>
   <si>
+    <t xml:space="preserve">atc1_medreq_fhir_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optional – FHIR ID of ATC1</t>
+  </si>
+  <si>
     <t xml:space="preserve">mrp_proxy_type</t>
   </si>
   <si>
@@ -134,6 +140,12 @@
   </si>
   <si>
     <t xml:space="preserve">optional – Code of the proxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrp_proxy_fhir_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optional – FHIR ID of the proxy</t>
   </si>
   <si>
     <t xml:space="preserve">input_file_processed_content_hash</t>
@@ -708,7 +720,8 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="1" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="6" t="s">
@@ -733,20 +746,40 @@
       <c r="B23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="6" t="s">
         <v>39</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-    </row>
-    <row r="1048328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+    </row>
     <row r="1048330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
feat: add non-FHIR pseudonym rules refs #1264
</commit_message>
<xml_diff>
--- a/R-dataprocessor/submodules/Dataprocessor_Submodules_Table_Description.xlsx
+++ b/R-dataprocessor/submodules/Dataprocessor_Submodules_Table_Description.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="47">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -76,6 +76,9 @@
     <t xml:space="preserve">COLUMN_TYPE</t>
   </si>
   <si>
+    <t xml:space="preserve">PSEUDONYMIZATION_RULE</t>
+  </si>
+  <si>
     <t xml:space="preserve"># Table to store for which Encounters and which Medication Analyses the MRP calculation is completed.</t>
   </si>
   <si>
@@ -88,10 +91,16 @@
     <t xml:space="preserve">FHIR ID of the associated institution contact</t>
   </si>
   <si>
+    <t xml:space="preserve">cryptoHash</t>
+  </si>
+  <si>
     <t xml:space="preserve">mrp_calculation_type</t>
   </si>
   <si>
     <t xml:space="preserve">Type of MRP (name of the submodule which has calculated the MRP e.g. “Drug_Disease”, “Drug_Drug”, “Drug_DrugGoup”, “Drug_Kidney”)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep</t>
   </si>
   <si>
     <t xml:space="preserve">meda_id</t>
@@ -367,34 +376,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -540,12 +549,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5234375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="98.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="56.44"/>
   </cols>
   <sheetData>
@@ -626,153 +636,204 @@
       <c r="D12" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="E12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="1"/>
       <c r="XFD12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="F13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
       <c r="B17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="F17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
       <c r="B19" s="6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
       <c r="B20" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
       <c r="B21" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E23" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F23" s="1"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>